<commit_message>
Per-cycle QE lead report: inputs taken, artifacts produced, risks, go/no-go and sign-off; in UI, downloads and demo-artifacts
Co-Authored-By: Devin AI <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/agentic-qe-mvp/demo-artifacts/flow-1-baseline-CYC-1/08-report/CYC-1-cycle-report.xlsx
+++ b/agentic-qe-mvp/demo-artifacts/flow-1-baseline-CYC-1/08-report/CYC-1-cycle-report.xlsx
@@ -161,7 +161,7 @@
     <t>sri465inno/uc-agentic-quality-engineering@demo/commission-engine (df5203e)</t>
   </si>
   <si>
-    <t>Pulled live from GitHub: git clone of sri465inno/uc-agentic-quality-engineering@demo/commission-engine (df5203e) at 2026-09-28T21:39:39.079Z</t>
+    <t>Pulled live from GitHub: git clone of sri465inno/uc-agentic-quality-engineering@demo/commission-engine (df5203e) at 2026-09-28T21:43:24.968Z</t>
   </si>
   <si>
     <t>ID</t>
@@ -913,7 +913,7 @@
     <t>Priya Shah</t>
   </si>
   <si>
-    <t>2026-09-28T21:39:40.127Z</t>
+    <t>2026-09-28T21:43:25.867Z</t>
   </si>
   <si>
     <t>14 requirements approved; 0 excluded; 1 conflict(s) resolved</t>
@@ -3231,7 +3231,7 @@
         <v>224</v>
       </c>
       <c r="E3" s="2">
-        <v>244</v>
+        <v>232</v>
       </c>
       <c r="F3" s="2"/>
     </row>
@@ -3249,7 +3249,7 @@
         <v>224</v>
       </c>
       <c r="E4" s="2">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="F4" s="2"/>
     </row>
@@ -3267,7 +3267,7 @@
         <v>224</v>
       </c>
       <c r="E5" s="2">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F5" s="2"/>
     </row>
@@ -3303,7 +3303,7 @@
         <v>224</v>
       </c>
       <c r="E7" s="2">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F7" s="2"/>
     </row>
@@ -3321,7 +3321,7 @@
         <v>225</v>
       </c>
       <c r="E8" s="2">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F8" s="2"/>
     </row>
@@ -3339,7 +3339,7 @@
         <v>224</v>
       </c>
       <c r="E9" s="2">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="F9" s="2"/>
     </row>
@@ -3375,7 +3375,7 @@
         <v>224</v>
       </c>
       <c r="E11" s="2">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F11" s="2"/>
     </row>
@@ -3393,7 +3393,7 @@
         <v>224</v>
       </c>
       <c r="E12" s="2">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F12" s="2"/>
     </row>
@@ -3411,7 +3411,7 @@
         <v>224</v>
       </c>
       <c r="E13" s="2">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F13" s="2"/>
     </row>
@@ -3449,7 +3449,7 @@
         <v>224</v>
       </c>
       <c r="E15" s="2">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F15" s="2"/>
     </row>
@@ -3467,7 +3467,7 @@
         <v>224</v>
       </c>
       <c r="E16" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F16" s="2"/>
     </row>

</xml_diff>

<commit_message>
agentic-qe-mvp: type of testing steers the agents; advisory review agent before human review
Co-Authored-By: Devin AI <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/agentic-qe-mvp/demo-artifacts/flow-1-baseline-CYC-1/08-report/CYC-1-cycle-report.xlsx
+++ b/agentic-qe-mvp/demo-artifacts/flow-1-baseline-CYC-1/08-report/CYC-1-cycle-report.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="629" uniqueCount="352">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="643" uniqueCount="364">
   <si>
     <t>Metric</t>
   </si>
@@ -161,7 +161,7 @@
     <t>sri465inno/uc-agentic-quality-engineering@demo/commission-engine (df5203e)</t>
   </si>
   <si>
-    <t>Pulled live from GitHub: git clone of sri465inno/uc-agentic-quality-engineering@demo/commission-engine (df5203e) at 2026-09-28T21:43:24.968Z</t>
+    <t>Pulled live from GitHub: git clone of sri465inno/uc-agentic-quality-engineering@demo/commission-engine (df5203e) at 2026-09-29T17:20:27.149Z</t>
   </si>
   <si>
     <t>ID</t>
@@ -913,7 +913,7 @@
     <t>Priya Shah</t>
   </si>
   <si>
-    <t>2026-09-28T21:43:25.867Z</t>
+    <t>2026-09-29T17:20:28.339Z</t>
   </si>
   <si>
     <t>14 requirements approved; 0 excluded; 1 conflict(s) resolved</t>
@@ -1003,6 +1003,21 @@
     <t>input-normalisation.md</t>
   </si>
   <si>
+    <t>input-review</t>
+  </si>
+  <si>
+    <t>Input review before the human gate</t>
+  </si>
+  <si>
+    <t>What the review agent checks in the project inputs and how it words its suggestions for the reviewer.</t>
+  </si>
+  <si>
+    <t>review-agent</t>
+  </si>
+  <si>
+    <t>input-review.md</t>
+  </si>
+  <si>
     <t>test-case-authoring</t>
   </si>
   <si>
@@ -1018,6 +1033,21 @@
     <t>test-case-authoring.md</t>
   </si>
   <si>
+    <t>testing-regression</t>
+  </si>
+  <si>
+    <t>Regression pack</t>
+  </si>
+  <si>
+    <t>Steers the design and execution agents to keep and re-run the full pack so nothing that worked before breaks.</t>
+  </si>
+  <si>
+    <t>testcases, scripts, execution</t>
+  </si>
+  <si>
+    <t>testing-regression.md</t>
+  </si>
+  <si>
     <t>traceability-handover</t>
   </si>
   <si>
@@ -1060,6 +1090,9 @@
     <t>statements: delivered; gaps: delivered; conflicts: delivered</t>
   </si>
   <si>
+    <t>suggestions: delivered</t>
+  </si>
+  <si>
     <t>Requirements repository agent</t>
   </si>
   <si>
@@ -1078,22 +1111,25 @@
     <t>Test case agent</t>
   </si>
   <si>
-    <t>incremental-merge, test-case-authoring, traceability-handover</t>
-  </si>
-  <si>
-    <t>functional: delivered; nonFunctional: delivered</t>
+    <t>incremental-merge, test-case-authoring, testing-regression, traceability-handover</t>
+  </si>
+  <si>
+    <t>functional: delivered; nonFunctional: delivered; regressionPack: delivered</t>
   </si>
   <si>
     <t>Automation script agent</t>
   </si>
   <si>
-    <t>automation-script-conventions, incremental-merge, traceability-handover</t>
+    <t>automation-script-conventions, incremental-merge, testing-regression, traceability-handover</t>
   </si>
   <si>
     <t>specs: delivered</t>
   </si>
   <si>
     <t>Execution agent (Playwright, real run)</t>
+  </si>
+  <si>
+    <t>testing-regression, traceability-handover</t>
   </si>
   <si>
     <t>results: delivered</t>
@@ -1687,7 +1723,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -1833,6 +1869,40 @@
         <v>323</v>
       </c>
     </row>
+    <row r="9" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>324</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>333</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -1841,7 +1911,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
@@ -1853,155 +1923,169 @@
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>324</v>
+        <v>334</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>325</v>
+        <v>335</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>326</v>
+        <v>336</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>327</v>
+        <v>337</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>328</v>
+        <v>338</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>329</v>
+        <v>339</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>330</v>
+        <v>340</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>331</v>
+        <v>341</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>109</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
-        <v>333</v>
-      </c>
+        <v>342</v>
+      </c>
+    </row>
+    <row r="3" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B3" s="2" t="s">
-        <v>319</v>
+        <v>314</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>331</v>
+        <v>341</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>109</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>334</v>
+        <v>343</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>335</v>
+        <v>344</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>336</v>
+        <v>329</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>331</v>
+        <v>341</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>109</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>337</v>
+        <v>345</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>338</v>
+        <v>346</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>339</v>
+        <v>347</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>331</v>
+        <v>341</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>109</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>340</v>
+        <v>348</v>
       </c>
     </row>
     <row r="6" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
+        <v>349</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>341</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>342</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>331</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>109</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
     </row>
     <row r="7" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>344</v>
+        <v>352</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>319</v>
+        <v>353</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>331</v>
+        <v>341</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>109</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>345</v>
+        <v>354</v>
       </c>
     </row>
     <row r="8" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>346</v>
+        <v>355</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>347</v>
+        <v>356</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>331</v>
+        <v>341</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>109</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>348</v>
+        <v>357</v>
       </c>
     </row>
     <row r="9" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>349</v>
+        <v>358</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>350</v>
+        <v>359</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>331</v>
+        <v>341</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>109</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>351</v>
+        <v>360</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>363</v>
       </c>
     </row>
   </sheetData>
@@ -3213,7 +3297,7 @@
         <v>224</v>
       </c>
       <c r="E2" s="2">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F2" s="2"/>
     </row>
@@ -3231,7 +3315,7 @@
         <v>224</v>
       </c>
       <c r="E3" s="2">
-        <v>232</v>
+        <v>219</v>
       </c>
       <c r="F3" s="2"/>
     </row>
@@ -3249,7 +3333,7 @@
         <v>224</v>
       </c>
       <c r="E4" s="2">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F4" s="2"/>
     </row>
@@ -3267,7 +3351,7 @@
         <v>224</v>
       </c>
       <c r="E5" s="2">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F5" s="2"/>
     </row>
@@ -3285,7 +3369,7 @@
         <v>224</v>
       </c>
       <c r="E6" s="2">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F6" s="2"/>
     </row>
@@ -3339,7 +3423,7 @@
         <v>224</v>
       </c>
       <c r="E9" s="2">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="F9" s="2"/>
     </row>
@@ -3357,7 +3441,7 @@
         <v>224</v>
       </c>
       <c r="E10" s="2">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F10" s="2"/>
     </row>
@@ -3375,7 +3459,7 @@
         <v>224</v>
       </c>
       <c r="E11" s="2">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F11" s="2"/>
     </row>
@@ -3393,7 +3477,7 @@
         <v>224</v>
       </c>
       <c r="E12" s="2">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F12" s="2"/>
     </row>
@@ -3411,7 +3495,7 @@
         <v>224</v>
       </c>
       <c r="E13" s="2">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F13" s="2"/>
     </row>
@@ -3449,7 +3533,7 @@
         <v>224</v>
       </c>
       <c r="E15" s="2">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F15" s="2"/>
     </row>

</xml_diff>